<commit_message>
Synchronise verified evidence PDF links across dataset releases
</commit_message>
<xml_diff>
--- a/data/HEART_L4_Risk_Cards.xlsx
+++ b/data/HEART_L4_Risk_Cards.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Cards" sheetId="1" r:id="R577fda7750e24912"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="2" r:id="R7ebe168b85474169"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" r:id="Rac947a17c86d44c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Cards" sheetId="1" r:id="R1c5dc50556e54277"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Dictionary" sheetId="2" r:id="R10c4c8edbb75437a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Validation" sheetId="3" r:id="R38c25f830f8741a1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -542,7 +542,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V2" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W2" s="9" t="str">
         <x:v>… external changes to the system – such as the introduction of new agents or a distributional shift – can cause phase transitions, where the …</x:v>
@@ -626,7 +626,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V3" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W3" s="9" t="str">
         <x:v>… 2017; Sato et al., 2002; Vlatakis-Gkaragkounis et al., 2023), but can become the norm as the number of agents increases (Bielawski et al., 2021 …</x:v>
@@ -710,7 +710,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V4" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W4" s="9" t="str">
         <x:v>… arise from the interactions between agents, as each agent’s actions affect the environment and the behaviour of other agents, which in turn affect their …</x:v>
@@ -878,7 +878,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V6" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W6" s="9" t="str">
         <x:v>… Kay et al., 2024) of both other agents (Ju et al., 2024) and humans (see Case Study 7 and Section 3.1) Another increasingly important …</x:v>
@@ -962,7 +962,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V7" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W7" s="9" t="str">
         <x:v>… convergence to an optimal policy is guaranteed under modest conditions, but in the (mixed-motive) case of multiple agents, this same learning rule can lead …</x:v>
@@ -1046,7 +1046,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V8" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W8" s="9" t="str">
         <x:v>… massive collective resources of individual low- resourced actors, chained into an attack that breaks the assumptions of bandwidth constraints on a single well-resourced agent.</x:v>
@@ -1130,7 +1130,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V9" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W9" s="9" t="str">
         <x:v>… often arise from the interactions between agents, as each agent’s actions affect the environment and the behaviour of other agents, which in turn affect …</x:v>
@@ -1214,7 +1214,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V10" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W10" s="9" t="str">
         <x:v>… is especially concerning since they may operate inscrutably due to the speed, scale, complexity, or subtlety of their actions.17 Warnings of this possibility have …</x:v>
@@ -1382,7 +1382,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V12" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W12" s="9" t="str">
         <x:v>A closely related risk is the possibility of multiple agents combining different affordances to overcome safeguards, for which there is already preliminary evidence (Jones …</x:v>
@@ -1466,7 +1466,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V13" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W13" s="9" t="str">
         <x:v>… it has been critical to the success of superhuman systems, such as the use of self-play in algorithms like AlphaGo (Silver et al., 2016).</x:v>
@@ -1550,7 +1550,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V14" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W14" s="9" t="str">
         <x:v>… that when agents attempt to come to an agreement despite diverging interests, information asymmetries can lead to bargaining inef- ficiencies (Myerson &amp; Satterthwaite, 1983).</x:v>
@@ -1634,7 +1634,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V15" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W15" s="9" t="str">
         <x:v>… evolution selected for certain conflict-prone dispostions in humans, such as vengefulness, aggression, risk-seeking, selfishness, dishon- esty, deception, and spitefulness towards out-groups (Grafen, 1990; Han …</x:v>
@@ -1884,7 +1884,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V18" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W18" s="9" t="str">
         <x:v>… settings since the ability of agents to cooperate depends not only on the ability to coordinate on one of many arbitrary conventions (which might …</x:v>
@@ -1968,7 +1968,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V19" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W19" s="9" t="str">
         <x:v>… common-interest (and mixed-motive) settings often allow a vast number of mutually incompatible solutions (Schelling, 1980), which is worsened in partially observable environments (Bernstein et …</x:v>
@@ -2052,7 +2052,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V20" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W20" s="9" t="str">
         <x:v>In these settings, AI agents must solve the problem of ‘zero-shot’ (or, more generally, ‘few-shot’) coordination (Emmons et al., 2022; Hu et al., 2020 …</x:v>
@@ -2304,7 +2304,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V23" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W23" s="9" t="str">
         <x:v>… can introduce new attack vectors in multimodal models as well as expand the scope of the previous attacks, ranging from jailbreaking to poisoning [13].</x:v>
@@ -2640,7 +2640,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V27" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W27" s="9" t="str">
         <x:v>… effectively removes the human from the loop, which could prove disastrous in high-stakes contexts (e.g., a false positive in a nuclear sub- marine’s warning …</x:v>
@@ -2724,7 +2724,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V28" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W28" s="9" t="str">
         <x:v>As AI models and systems gain autonomy, the ability of humans to oversee and intervene in decision-making processes diminishes.</x:v>
@@ -2892,7 +2892,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V30" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W30" s="9" t="str">
         <x:v>Profound negative long-term changes to social structures, cultural norms, and human relationships that may be difficult or impossible to reverse.</x:v>
@@ -3562,7 +3562,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V38" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W38" s="9" t="str">
         <x:v>An AI system may have the ability to bypass a sandboxed environment in which it is trained or evaluated.</x:v>
@@ -3646,7 +3646,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V39" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W39" s="9" t="str">
         <x:v>… al., 2023b) and ‘illusory’ attacks (Franzmeyer et al., 2023), which are black-box undetectable and can even be hidden using white-box undetectable encrypted backdoors (Draguns …</x:v>
@@ -3814,7 +3814,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V41" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W41" s="9" t="str">
         <x:v>AI models and systems that appear aligned with human goals during development may behave unpredictably or dangerously once deployed</x:v>
@@ -3898,7 +3898,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V42" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W42" s="9" t="str">
         <x:v>AI models and systems that appear aligned with human goals during development may behave unpredictably or dangerously once deployed</x:v>
@@ -3986,7 +3986,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V43" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W43" s="9" t="str">
         <x:v>This harms both the user and the provider, as the provider is exposed to increased legal liability due to the model’s actions.</x:v>
@@ -4238,7 +4238,7 @@
         <x:v>10.48550/arXiv.1511.03246</x:v>
       </x:c>
       <x:c r="V46" s="9" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.1511.03246</x:v>
+        <x:v>https://arxiv.org/pdf/1511.03246</x:v>
       </x:c>
       <x:c r="W46" s="9" t="str">
         <x:v>… properties, which may make it less likely to abide by any built-in rules or regulations and to instead pursue its own goals possibly to …</x:v>
@@ -4820,7 +4820,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V53" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W53" s="9" t="str">
         <x:v>The human evaluator can rate incorrect outputs positively or similar to correct outputs.</x:v>
@@ -4986,7 +4986,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V55" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W55" s="9" t="str">
         <x:v>AI systems can achieve user-specified tasks in undesirable ways unless they are specified carefully and in enough detail.</x:v>
@@ -5070,7 +5070,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V56" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W56" s="9" t="str">
         <x:v>… specification gaming (such as sycophancy in LLMs) can, if left unchecked, enable the model to generalize to more sophisticated behavior such as reward tampering …</x:v>
@@ -5154,7 +5154,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V57" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W57" s="9" t="str">
         <x:v>… learns from feedback for performing actions in an environment (e.g., rein- forcement learning), intervenes on the mechanisms that determine its training reward or loss.</x:v>
@@ -5238,7 +5238,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V58" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W58" s="9" t="str">
         <x:v>… when it is useful (i.e., predictive) to do so.51 While it might not be helpful to describe individual narrow AI tools as having goals …</x:v>
@@ -5488,7 +5488,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V61" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W61" s="9" t="str">
         <x:v>Whether the risk originates from malicious intent or is an unintended consequence of legitimate task objectives</x:v>
@@ -5824,7 +5824,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V65" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W65" s="9" t="str">
         <x:v>The human evaluator can rate incorrect outputs positively or similar to correct outputs.</x:v>
@@ -6076,7 +6076,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V68" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W68" s="9" t="str">
         <x:v>When multiple actors are involved in AI development and deployment, it becomes difficult to assign responsibility for harm, complicating accountability.</x:v>
@@ -6416,7 +6416,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V72" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W72" s="9" t="str">
         <x:v>Benefits/entitlements loss - Denial or or loss of access to welfare benefits, pensions, housing, etc due to the malfunction, use or abuse of a …</x:v>
@@ -6582,7 +6582,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V74" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W74" s="9" t="str">
         <x:v>AI systems can undermine human autonomy, if they allow for habitually trusting the AI’s suggestions without sufficient exercising of human agency.</x:v>
@@ -6930,7 +6930,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V78" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W78" s="9" t="str">
         <x:v>AI-based content moderation algorithms, while intended to filter harmful con- tent, can perpetuate biases.</x:v>
@@ -7278,7 +7278,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V82" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W82" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -7542,7 +7542,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V85" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W85" s="9" t="str">
         <x:v>The large-scale erosion or violation of fundamental human rights and freedoms.</x:v>
@@ -7710,7 +7710,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V87" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W87" s="9" t="str">
         <x:v>When multiple actors are involved in AI development and deployment, it becomes difficult to assign responsibility for harm, complicating accountability.</x:v>
@@ -9006,7 +9006,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V102" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W102" s="9" t="str">
         <x:v>They can also involve the imitation of speech or body movements of real people.</x:v>
@@ -9094,7 +9094,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V103" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W103" s="9" t="str">
         <x:v>Impersonation/identity theft - Theft of an individual, group or organisation’s identity by a third-party in order to defraud, mock or otherwise harm them.</x:v>
@@ -9356,7 +9356,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V106" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W106" s="9" t="str">
         <x:v>GPAIs can be misused for the automated generation of content personalized to target select individuals based on their weak spots [30].</x:v>
@@ -9698,7 +9698,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V110" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W110" s="9" t="str">
         <x:v>These threats might target humans directly (such as the revelation of private information extracted by advanced AI surveillance tools), or other AI systems that …</x:v>
@@ -9782,7 +9782,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V111" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W111" s="9" t="str">
         <x:v>Harassment/abuse/intimidation - Online behaviour, including sexual harassment, that makes an individual or group feel alarmed or threatened.</x:v>
@@ -9954,7 +9954,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V113" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W113" s="9" t="str">
         <x:v>GPAI tools can be used in automation and scaling of influence campaigns [178].</x:v>
@@ -10128,7 +10128,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V115" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W115" s="9" t="str">
         <x:v>Electoral interference - Generation of false or misleading information that can interrupt or mislead voters and/or undermine trust in electoral processes.</x:v>
@@ -10302,7 +10302,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V117" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W117" s="9" t="str">
         <x:v>… manipulation - Use or misuse of personal data to target individuals’ interests, personalities and vulnerabilities with tailored political messages via micro-advertising or deepfakes/synthetic media.</x:v>
@@ -10990,7 +10990,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V125" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W125" s="9" t="str">
         <x:v>Data Exfiltration goes beyond revealing private information, and involves illicitly obtaining the training data used to build a model that may be sensitive or …</x:v>
@@ -12628,7 +12628,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V144" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W144" s="9" t="str">
         <x:v>AI models and systems may grant governments or corporations increased monitoring over individuals.</x:v>
@@ -12796,7 +12796,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V146" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W146" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -12964,7 +12964,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V148" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W148" s="9" t="str">
         <x:v>In particular, less confident users (or users in emotional distress) can be more prone to “overtrust” a system [219].</x:v>
@@ -13048,7 +13048,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V149" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W149" s="9" t="str">
         <x:v>Alienation/isolation - An individual’s or group’s feeling of lack of connection with those around as a result of technology use or misuse.</x:v>
@@ -13556,7 +13556,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V155" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W155" s="9" t="str">
         <x:v>Dehumanisation/objectification - Use or misuse of a technology system to depict and/or treat people as not human, less than human, or as objects.</x:v>
@@ -13728,7 +13728,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V157" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W157" s="9" t="str">
         <x:v>AI-based content moderation algorithms, while intended to filter harmful con- tent, can perpetuate biases.</x:v>
@@ -15120,7 +15120,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V173" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W173" s="9" t="str">
         <x:v>… in AI models can be affected by and continue to exhibit previously encountered biases in their decision-making, even after they stop using the models …</x:v>
@@ -15384,7 +15384,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V176" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W176" s="9" t="str">
         <x:v>Dataset bias may be unintentionally amplified [60] where the outputs of the AI model trained on a dataset are more biased than the dataset …</x:v>
@@ -15900,7 +15900,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2503.05731</x:v>
       </x:c>
       <x:c r="V182" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2503.05731</x:v>
+        <x:v>https://arxiv.org/pdf/2503.05731</x:v>
       </x:c>
       <x:c r="W182" s="9" t="str">
         <x:v>They may also enable, encourage, or endorse actions for which self-harm is not the desired result (e.g., smoking cigarettes or participating in extreme sports).</x:v>
@@ -16076,7 +16076,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2503.05731</x:v>
       </x:c>
       <x:c r="V184" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2503.05731</x:v>
+        <x:v>https://arxiv.org/pdf/2503.05731</x:v>
       </x:c>
       <x:c r="W184" s="9" t="str">
         <x:v>Unacceptable responses will enable, encourage, or endorse acts of intentional self-harm: • Suicide.</x:v>
@@ -16252,7 +16252,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2503.05731</x:v>
       </x:c>
       <x:c r="V186" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2503.05731</x:v>
+        <x:v>https://arxiv.org/pdf/2503.05731</x:v>
       </x:c>
       <x:c r="W186" s="9" t="str">
         <x:v>Suicide and Self-Harm Acceptable responses may describe or provide information about suicide and self-harm.</x:v>
@@ -16340,7 +16340,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2503.05731</x:v>
       </x:c>
       <x:c r="V187" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2503.05731</x:v>
+        <x:v>https://arxiv.org/pdf/2503.05731</x:v>
       </x:c>
       <x:c r="W187" s="9" t="str">
         <x:v>Suicide and Self-Harm Acceptable responses may describe or provide information about suicide and self-harm.</x:v>
@@ -16428,7 +16428,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V188" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W188" s="9" t="str">
         <x:v>Generative models can create illegal, harmful, or discriminatory content [196], such as sexual abuse material, at scale.</x:v>
@@ -16604,7 +16604,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V190" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W190" s="9" t="str">
         <x:v>Create sexual explicit material using an adult person’s likeness</x:v>
@@ -16862,7 +16862,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V193" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W193" s="9" t="str">
         <x:v>Harassment/abuse/intimidation - Online behaviour, including sexual harassment, that makes an individual or group feel alarmed or threatened.</x:v>
@@ -16950,7 +16950,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V194" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W194" s="9" t="str">
         <x:v>Create child sexual explicit material</x:v>
@@ -17550,7 +17550,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V201" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W201" s="9" t="str">
         <x:v>Advanced GPAI systems can create advertisements tailored to individual recip- ients, exploiting the biases and irrational beliefs of each recipient.</x:v>
@@ -17634,7 +17634,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V202" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W202" s="9" t="str">
         <x:v>… technology system to covertly alter user beliefs and behaviour using nudging, dark patterns and/or other opaque techniques, resulting in potential erosion of privacy, addiction …</x:v>
@@ -17806,7 +17806,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V204" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W204" s="9" t="str">
         <x:v>Benign intermediate for harmful end objective</x:v>
@@ -18150,7 +18150,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V208" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W208" s="9" t="str">
         <x:v>AI-based content moderation algorithms, while intended to filter harmful con- tent, can perpetuate biases.</x:v>
@@ -18234,7 +18234,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V209" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W209" s="9" t="str">
         <x:v>Coercion/manipulation - Use of a technology system to covertly alter user beliefs and behaviour using nudging, dark patterns and/or other opaque techniques, resulting in …</x:v>
@@ -18318,7 +18318,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V210" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W210" s="9" t="str">
         <x:v>AI models and systems might develop goals that diverge from human intentions.</x:v>
@@ -18402,7 +18402,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V211" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W211" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -18658,7 +18658,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V214" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W214" s="9" t="str">
         <x:v>Refine outputs to target individuals with tailored attacks</x:v>
@@ -18742,7 +18742,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V215" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W215" s="9" t="str">
         <x:v>… that models trained on human data – such as being pre-trained on human-written text or fine-tuned on human feedback – can exhibit human biases.</x:v>
@@ -18910,7 +18910,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V217" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W217" s="9" t="str">
         <x:v>AI systems with natural-language outputs can tend to give answers that appear plausible or that users prefer [149] but are factually incorrect.</x:v>
@@ -18994,7 +18994,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V218" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W218" s="9" t="str">
         <x:v>AI models and systems that lack moral reasoning capabilities may make decisions that are unethical or harmful.</x:v>
@@ -19082,7 +19082,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V219" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W219" s="9" t="str">
         <x:v>Increased competition - The inappropriate or unethical use of technology to gain market share.</x:v>
@@ -19250,7 +19250,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V221" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W221" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -19678,7 +19678,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V226" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W226" s="9" t="str">
         <x:v>This bias can lead to an imbalance, where easier-to-measure values dominate the evaluation process, while other important values are underrepresented.</x:v>
@@ -19846,7 +19846,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V228" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W228" s="9" t="str">
         <x:v>The dominance of specific AI models could lead to a lack of diversity in approaches, amplifying systemic risks if these models fail.</x:v>
@@ -20016,7 +20016,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V230" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W230" s="9" t="str">
         <x:v>This can lead to a false sense of safety and trust due to a lack of understanding of the model’s limitations.</x:v>
@@ -20268,7 +20268,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V233" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W233" s="9" t="str">
         <x:v>… where an AI system appears to be pursuing the intended objective in training, but does not generalize to pursuing this objective in out-of-distribution settings …</x:v>
@@ -20696,7 +20696,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V238" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W238" s="9" t="str">
         <x:v>… Adoption of extreme political, social, or religious ideals and aspirations due to the nature or misuse of an algorithmic system, potentially resulting in abuse …</x:v>
@@ -21392,7 +21392,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V246" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W246" s="9" t="str">
         <x:v>Harassment/abuse/intimidation - Online behaviour, including sexual harassment, that makes an individual or group feel alarmed or threatened.</x:v>
@@ -21740,7 +21740,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V250" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W250" s="9" t="str">
         <x:v>… to aid in the creation of weapons, such as chemical, biological, radiological, and nuclear (CBRN) weapons, or augment the abilities of existing weapons, such …</x:v>
@@ -22000,7 +22000,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V253" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W253" s="9" t="str">
         <x:v>Models used for drug discovery, such as drug-target affinity prediction models, can be used to identify or develop dangerous toxins.</x:v>
@@ -22088,7 +22088,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V254" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W254" s="9" t="str">
         <x:v>AI capabilities that could be deliberately weaponized for destructive purposes.</x:v>
@@ -22172,7 +22172,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V255" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W255" s="9" t="str">
         <x:v>AI can be used to enhance pathogens, making them more lethal or resistant to treatments.</x:v>
@@ -22520,7 +22520,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V259" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W259" s="9" t="str">
         <x:v>This type of automation allows attackers to expand the scale of their operations at a low cost, increasing the impact of their actions.</x:v>
@@ -22696,7 +22696,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V261" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W261" s="9" t="str">
         <x:v>… both immediate operational hazards, such as exposure incidents or containment failures during the automated handling of radioactive materials, and broader security concerns regarding the …</x:v>
@@ -22864,7 +22864,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V263" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W263" s="9" t="str">
         <x:v>Powerful AI technologies may fall into the hands of terrorists.</x:v>
@@ -23296,7 +23296,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V268" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W268" s="9" t="str">
         <x:v>… the creation of weapons, such as chemical, biological, radiological, and nuclear (CBRN) weapons, or augment the abilities of existing weapons, such as providing autonomous …</x:v>
@@ -23894,7 +23894,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V275" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W275" s="9" t="str">
         <x:v>Loss of creativity/critical thinking - Devaluation and/or deterioration of human creativity, artistic ex- pression, imagination, critical thinking or problem-solving skills.</x:v>
@@ -24656,7 +24656,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V284" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W284" s="9" t="str">
         <x:v>… or containment failures during the automated handling of radioactive materials, and broader security concerns regarding the potential misuse of AI systems in nuclear research.</x:v>
@@ -24740,7 +24740,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V285" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W285" s="9" t="str">
         <x:v>Excessive reliance on specific AI providers can lead to vulnerabilities due to lack of alternatives or interoperability.</x:v>
@@ -25164,7 +25164,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V290" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W290" s="9" t="str">
         <x:v>The erosion of democratic processes and public trust in social/political institutions.</x:v>
@@ -25330,7 +25330,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V292" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W292" s="9" t="str">
         <x:v>Large-scale influence on communication and information systems, and epistemic processes more generally.</x:v>
@@ -25586,7 +25586,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V295" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W295" s="9" t="str">
         <x:v>AI-based surveillance and manipulation could be used to maintain global totalitarian regimes.</x:v>
@@ -26178,7 +26178,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V302" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W302" s="9" t="str">
         <x:v>Outsourcing tasks like data labeling to low-income countries can perpetuate inequality.</x:v>
@@ -26430,7 +26430,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V305" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W305" s="9" t="str">
         <x:v>… Societal instability in the form of strikes, demonstrations and other types of civil unrest caused by loss of jobs to technology, unfair algorithmic outcomes …</x:v>
@@ -26598,7 +26598,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V307" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W307" s="9" t="str">
         <x:v>Training and deploying large models require substantial energy expenditure.</x:v>
@@ -26682,7 +26682,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V308" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W308" s="9" t="str">
         <x:v>… - Over-expansion of technology infrastructure, or inadequate alignment of technology with sustainable practices, leading to deforestation, habitat destruction, and fragmentation and loss of biodiversity.</x:v>
@@ -26934,7 +26934,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V311" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W311" s="9" t="str">
         <x:v>… landfill - Excessive disposal of electrical or electronic equipment leading to ecological/biodiversity damage, and disrupting the livelihoods and eroding the rights of local communities.</x:v>
@@ -27106,7 +27106,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V313" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W313" s="9" t="str">
         <x:v>… (e.g., sexualization of photos of women [87] in the case of image generation models) or they can generate toxic, misleading, or violent data (e.g. …</x:v>
@@ -27616,7 +27616,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V319" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W319" s="9" t="str">
         <x:v>Designers and operators of AI may face conflicting objectives that compromise safety.</x:v>
@@ -27784,7 +27784,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V321" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W321" s="9" t="str">
         <x:v>Heavy reliance on AI in critical sectors like finance or healthcare can exacerbate issues related to size, speed, interconnectivity, and complexity of the system.</x:v>
@@ -27868,7 +27868,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V322" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W322" s="9" t="str">
         <x:v>Heavy reliance on AI in critical sectors like finance or healthcare can exacerbate issues related to size, speed, interconnectivity, and complexity of the system.</x:v>
@@ -28874,7 +28874,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V334" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W334" s="9" t="str">
         <x:v>The fast pace of AI development may outstrip regulatory and legal frameworks.</x:v>
@@ -29210,7 +29210,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V338" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W338" s="9" t="str">
         <x:v>As AI models and systems gain autonomy, the ability of humans to oversee and intervene in decision-making processes diminishes.</x:v>
@@ -29378,7 +29378,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V340" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W340" s="9" t="str">
         <x:v>When multiple actors are involved in AI development and deployment, it becomes difficult to assign responsibility for harm, complicating accountability.</x:v>
@@ -29462,7 +29462,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V341" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W341" s="9" t="str">
         <x:v>Interactions between different AI components can cause harm, but it may be difficult to pinpoint which components are the cause.</x:v>
@@ -29630,7 +29630,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V343" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W343" s="9" t="str">
         <x:v>The complex and rapidly evolving nature of AI makes them inherently difficult to govern effectively, leading to systemic regulatory and oversight failures.</x:v>
@@ -29714,7 +29714,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V344" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W344" s="9" t="str">
         <x:v>The complex and rapidly evolving nature of AI makes them inherently difficult to govern effectively, leading to systemic regulatory and oversight failures.</x:v>
@@ -29882,7 +29882,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V346" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W346" s="9" t="str">
         <x:v>For GPAIs or foundation models, risks emerge during training, prior to being repurposed and deployed in more specific AI systems or applications.</x:v>
@@ -29966,7 +29966,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V347" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W347" s="9" t="str">
         <x:v>… competitive situations, developers of general-purpose AI systems might cut corners on the safety evaluation of their GPAI model and instead spend more time and …</x:v>
@@ -30050,7 +30050,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V348" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W348" s="9" t="str">
         <x:v>Excessive reliance on specific AI providers can lead to vulnerabilities due to lack of alternatives or interoperability.</x:v>
@@ -30134,7 +30134,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V349" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W349" s="9" t="str">
         <x:v>The widespread use of common AI platforms can create centralized points of failure, making systems more vulnerable to disruptions or attacks</x:v>
@@ -30554,7 +30554,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V354" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W354" s="9" t="str">
         <x:v>… create such models (and continuing returns to scale) means that only well-resourced actors can create cutting- edge models (Epoch, 2023; Hoffmann et al., 2022 …</x:v>
@@ -30888,7 +30888,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V358" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W358" s="9" t="str">
         <x:v>Outsourcing tasks like data labeling to low-income countries can perpetuate inequality.</x:v>
@@ -31138,7 +31138,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V361" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W361" s="9" t="str">
         <x:v>The complex and rapidly evolving nature of AI makes them inherently difficult to govern effectively, leading to systemic regulatory and oversight failures.</x:v>
@@ -31636,7 +31636,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V367" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W367" s="9" t="str">
         <x:v>The tendency for humans to over-rely on AI models and systems, trusting their outputs without sufficient critical evaluation, which can lead to poor decision-making.</x:v>
@@ -31720,7 +31720,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V368" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W368" s="9" t="str">
         <x:v>The human evaluator can rate incorrect outputs positively or similar to correct outputs.</x:v>
@@ -31808,7 +31808,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V369" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W369" s="9" t="str">
         <x:v>AI models and systems could decide or influence important personal decisions.</x:v>
@@ -32058,7 +32058,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V372" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W372" s="9" t="str">
         <x:v>AI models and systems could decide or influence important personal decisions.</x:v>
@@ -32314,7 +32314,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V375" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W375" s="9" t="str">
         <x:v>AI systems can undermine human autonomy, if they allow for habitually trusting the AI’s suggestions without sufficient exercising of human agency.</x:v>
@@ -32398,7 +32398,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V376" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W376" s="9" t="str">
         <x:v>Auditors may not be able to address all of the specific safety, performance, or validation needs.</x:v>
@@ -32570,7 +32570,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V378" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W378" s="9" t="str">
         <x:v>Situational awareness in GPAI systems refers to the ability to understand its context, environment, and use this to inform action.</x:v>
@@ -32738,7 +32738,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V380" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W380" s="9" t="str">
         <x:v>… most basic form of this is when a benchmark is trans- lated to another language and then fed to the model as training data.</x:v>
@@ -32990,7 +32990,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V383" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W383" s="9" t="str">
         <x:v>… to measuring the performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in …</x:v>
@@ -33158,7 +33158,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V385" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W385" s="9" t="str">
         <x:v>Excessive reliance on specific AI providers can lead to vulnerabilities due to lack of alternatives or interoperability.</x:v>
@@ -33242,7 +33242,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V386" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W386" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -33326,7 +33326,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V387" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W387" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -33410,7 +33410,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V388" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W388" s="9" t="str">
         <x:v>Conflicts of interest can arise if there is no independence in the auditor selection process or if the auditors are closely associated with the …</x:v>
@@ -33494,7 +33494,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V389" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W389" s="9" t="str">
         <x:v>This can lead to a false sense of safety and trust due to a lack of understanding of the model’s limitations.</x:v>
@@ -33578,7 +33578,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V390" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W390" s="9" t="str">
         <x:v>… of test coverage by benchmarks on specific abilities of a model can obscure the model’s capabilities from both the developer and the user [160].</x:v>
@@ -33662,7 +33662,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V391" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W391" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -33746,7 +33746,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V392" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W392" s="9" t="str">
         <x:v>The capabilities of general-purpose AI systems can be difficult to measure, compared to the capabilities of more limited and fixed-purpose AI systems.</x:v>
@@ -33830,7 +33830,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V393" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W393" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -33914,7 +33914,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V394" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W394" s="9" t="str">
         <x:v>Benchmarks dedicated to measuring the performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and …</x:v>
@@ -34082,7 +34082,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V396" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W396" s="9" t="str">
         <x:v>… sufficient infrastructure, including the absence of quality control processes for collecting data, especially for high-stakes domains and benchmarks, can affect the quality and type …</x:v>
@@ -34250,7 +34250,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V398" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W398" s="9" t="str">
         <x:v>The capabilities of general-purpose AI systems can be difficult to measure, compared to the capabilities of more limited and fixed-purpose AI systems.</x:v>
@@ -34334,7 +34334,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V399" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W399" s="9" t="str">
         <x:v>Even minor modifications can lead to significant shifts in model performance, potentially affecting the reliability of model evaluations and comparisons.</x:v>
@@ -34500,7 +34500,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V401" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W401" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -34584,7 +34584,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V402" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W402" s="9" t="str">
         <x:v>As AI models and systems gain autonomy, the ability of humans to oversee and intervene in decision-making processes diminishes.</x:v>
@@ -34668,7 +34668,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V403" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W403" s="9" t="str">
         <x:v>This can lead to a false sense of safety and trust due to a lack of understanding of the model’s limitations.</x:v>
@@ -34920,7 +34920,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V406" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W406" s="9" t="str">
         <x:v>This can lead to the model learning to produce subtly incorrect or harmful outputs, such as code with software vulnerabilities, or politically biased information.</x:v>
@@ -35086,7 +35086,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V408" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W408" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -35170,7 +35170,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V409" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W409" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -35254,7 +35254,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V410" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W410" s="9" t="str">
         <x:v>… LLM-based evaluation is integrated into the training of a new model, the trained model could develop in a way that specifically finds and exploits …</x:v>
@@ -35506,7 +35506,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V413" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W413" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -35590,7 +35590,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V414" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W414" s="9" t="str">
         <x:v>… of human values learned by the model, and it is not known how these values evolve and transition across different stages of model training …</x:v>
@@ -35674,7 +35674,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V415" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W415" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -35846,7 +35846,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V417" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W417" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -36014,7 +36014,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V419" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W419" s="9" t="str">
         <x:v>Risk assessments can be conducted before deployment, and monitoring of AI models can occur as required throughout the deployment phase.</x:v>
@@ -36266,7 +36266,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V422" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W422" s="9" t="str">
         <x:v>Harm from AI often manifests subtly or over the long term, making it difficult to identify, measure, and address effectively.</x:v>
@@ -36350,7 +36350,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V423" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W423" s="9" t="str">
         <x:v>These instructions may contain explicit data-label pairs that can improve the model’s capabilities for the task.</x:v>
@@ -36684,7 +36684,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V427" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W427" s="9" t="str">
         <x:v>… of test coverage by benchmarks on specific abilities of a model can obscure the model’s capabilities from both the developer and the user [160].</x:v>
@@ -36768,7 +36768,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V428" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W428" s="9" t="str">
         <x:v>… relevant in self-evaluation tasks, where a model assesses the quality or persua- siveness [66] of its own outputs, or in model-based evaluations more broadly.</x:v>
@@ -36852,7 +36852,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V429" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W429" s="9" t="str">
         <x:v>… competitive situations, developers of general-purpose AI systems might cut corners on the safety evaluation of their GPAI model and instead spend more time and …</x:v>
@@ -36936,7 +36936,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V430" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W430" s="9" t="str">
         <x:v>… more and more kinds of information, AI agents could end up ‘polluting the epistemic commons’ (Huang &amp; Siddarth, 2023; Kay et al., 2024) of …</x:v>
@@ -37020,7 +37020,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V431" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W431" s="9" t="str">
         <x:v>… example, evaluations may miss certain capabilities that are difficult to assess, prohibitively costly to verify, or obscured by the model’s tendency to refuse responses …</x:v>
@@ -37104,7 +37104,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V432" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W432" s="9" t="str">
         <x:v>… fast operational speed of AI models and systems in competitive environments can lead to errors that are difficult to detect and correct in time.</x:v>
@@ -37272,7 +37272,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V434" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W434" s="9" t="str">
         <x:v>… in AI models that are easier to evaluate might be preferred for inclusion in evaluations over those that are more difficult to measure [13].</x:v>
@@ -37356,7 +37356,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V435" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W435" s="9" t="str">
         <x:v>… inclusive than can be justified due to a lack of knowledge of specific risks and how they can be tested, or a lack of …</x:v>
@@ -37444,7 +37444,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V436" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W436" s="9" t="str">
         <x:v>This can lead to a false sense of safety and trust due to a lack of understanding of the model’s limitations.</x:v>
@@ -37528,7 +37528,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V437" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W437" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -37612,7 +37612,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V438" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W438" s="9" t="str">
         <x:v>… performance of AI systems (e.g., on programming or math tasks) are more well-developed than those for assessing safety and harms in AI systems [234].</x:v>
@@ -37700,7 +37700,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V439" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W439" s="9" t="str">
         <x:v>Designers and operators of AI may face conflicting objectives that compromise safety.</x:v>
@@ -37784,7 +37784,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V440" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W440" s="9" t="str">
         <x:v>AI systems with natural-language outputs can tend to give answers that appear plausible or that users prefer [149] but are factually incorrect.</x:v>
@@ -38044,7 +38044,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V443" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W443" s="9" t="str">
         <x:v>… not perfectly reflect the representation of human values learned by the model, and it is not known how these values evolve and transition across …</x:v>
@@ -38296,7 +38296,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V446" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W446" s="9" t="str">
         <x:v>AI systems with natural-language outputs can tend to give answers that appear plausible or that users prefer [149] but are factually incorrect.</x:v>
@@ -38548,7 +38548,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V449" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W449" s="9" t="str">
         <x:v>Multi-turn persuasion can be more effective than single-turn persuasion attempts in altering the model’s stance [223].</x:v>
@@ -38632,7 +38632,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V450" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W450" s="9" t="str">
         <x:v>… the misuse, misinterpretation, or leakage of data, which can lead to erroneous conclusions or the unintentional dissemination of sensitive information, such as private patient …</x:v>
@@ -38800,7 +38800,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V452" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W452" s="9" t="str">
         <x:v>The difficulty in distinguishing synthetic content from authentic material adds to information risks.</x:v>
@@ -39048,7 +39048,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V455" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W455" s="9" t="str">
         <x:v>… lead to models producing false outputs given false information during the retrieval- augmentation process, despite only a relatively small amount of false informa- tion …</x:v>
@@ -39132,7 +39132,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V456" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W456" s="9" t="str">
         <x:v>AI models may generate false or misleading information due to their lack of capability in discerning truth.</x:v>
@@ -39216,7 +39216,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V457" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W457" s="9" t="str">
         <x:v>Historical revisionism - Deliberate or unintentional reinterpretation of established/orthodox historical events or accounts held by societies, communities, academics.</x:v>
@@ -39984,7 +39984,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V466" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W466" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -40072,7 +40072,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V467" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W467" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -40160,7 +40160,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V468" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W468" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -40248,7 +40248,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V469" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W469" s="9" t="str">
         <x:v>… develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s domain of expertise [205, 42].</x:v>
@@ -40592,7 +40592,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V473" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W473" s="9" t="str">
         <x:v>AI models and systems are vulnerable to manipulation through adversarial inputs.</x:v>
@@ -40844,7 +40844,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V476" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W476" s="9" t="str">
         <x:v>Over time, a user may develop unjustified trust in or dependence on the system, or rely on its advice for tasks outside the system’s …</x:v>
@@ -41096,7 +41096,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V479" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W479" s="9" t="str">
         <x:v>… easily become distracted by irrelevant provided information (such as “context” in LLMs), leading to a significant decrease in their performance after introducing irrelevant information.</x:v>
@@ -41180,7 +41180,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V480" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W480" s="9" t="str">
         <x:v>Catastrophic forgetting occurs when a model loses its ability to retain previously learned tasks (or factual information) after being trained on new ones.</x:v>
@@ -41932,7 +41932,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V489" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W489" s="9" t="str">
         <x:v>… be more likely to produce undesired or harmful outputs (as compared to the non-fine-tuned model), even if the fine-tuning was done with harmless and …</x:v>
@@ -42016,7 +42016,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V490" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W490" s="9" t="str">
         <x:v>Common manipulations applied on data in the context of AI models include defining the ground truth label and merging different data formats or sources.</x:v>
@@ -42268,7 +42268,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V493" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W493" s="9" t="str">
         <x:v>Public service delivery deterioration - Poor performance of a public technology system due to malfunc- tion, over-use, under-staffing etc, resulting in individuals, groups, or …</x:v>
@@ -42352,7 +42352,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V494" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W494" s="9" t="str">
         <x:v>Adversarial training can be affected by robust overfitting, where the model’s robustness on test data decreases during further training, particularly after the learning rate …</x:v>
@@ -42436,7 +42436,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V495" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W495" s="9" t="str">
         <x:v>Deployed AI systems can rely on physical sensors and data sources that may exhibit hardware drift and thus data distribution drift over time.</x:v>
@@ -42520,7 +42520,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V496" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W496" s="9" t="str">
         <x:v>… be more likely to produce undesired or harmful outputs (as compared to the non-fine-tuned model), even if the fine-tuning was done with harmless and …</x:v>
@@ -42688,7 +42688,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V498" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W498" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -42772,7 +42772,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V499" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W499" s="9" t="str">
         <x:v>As above, there are broadly two dimensions of technical failure modes: quality of data or input signal, and training performance.</x:v>
@@ -43022,7 +43022,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V502" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W502" s="9" t="str">
         <x:v>Data Exfiltration goes beyond revealing private information, and involves illicitly obtaining the training data used to build a model that may be sensitive or …</x:v>
@@ -43106,7 +43106,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V503" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W503" s="9" t="str">
         <x:v>… AI model easier to implement, such as finding adversarial examples, elicitation of dangerous capabilities, and extraction of confidential information present in the training data.</x:v>
@@ -43274,7 +43274,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V505" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W505" s="9" t="str">
         <x:v>Prompt Injections are a form of Adversarial Input that involve manipulating the text instructions given to a GenAI system (Liu et al., 2023).</x:v>
@@ -43616,7 +43616,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V509" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W509" s="9" t="str">
         <x:v>These modifications, which are often imperceptible to humans, exploit how the model makes decisions to produce errors (Wallace et al., 2019) and can be …</x:v>
@@ -43782,7 +43782,7 @@
         <x:v>10.48550/arXiv.2402.04247</x:v>
       </x:c>
       <x:c r="V511" s="9" t="str">
-        <x:v>https://icml.cc/virtual/2025/51008</x:v>
+        <x:v>https://arxiv.org/pdf/2402.04247</x:v>
       </x:c>
       <x:c r="W511" s="9" t="str">
         <x:v>Whether the risk originates from malicious intent or is an unintended consequence of legitimate task objectives</x:v>
@@ -43866,7 +43866,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V512" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W512" s="9" t="str">
         <x:v>Without careful planning and the appropriate safeguards, we may soon be entering a world overrun by increasingly competent and autonomous software agents, able to …</x:v>
@@ -44032,7 +44032,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V514" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W514" s="9" t="str">
         <x:v>… can introduce new attack vectors in multimodal models as well as expand the scope of the previous attacks, ranging from jailbreaking to poisoning [13].</x:v>
@@ -44116,7 +44116,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V515" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W515" s="9" t="str">
         <x:v>A jailbreak is a type of adversarial input to the model (during deployment) re- sulting in model behavior deviating from intended use.</x:v>
@@ -44284,7 +44284,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V517" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W517" s="9" t="str">
         <x:v>… can be exploited with minimal overhead, al- lowing attackers to control the model outputs in a targeted way with a high success rate [90].</x:v>
@@ -44368,7 +44368,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V518" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W518" s="9" t="str">
         <x:v>… in critical infrastructure, there may be common mode failures that begin with vulnerabilities or robustness issues in the underlying model architecture or training setup.</x:v>
@@ -44452,7 +44452,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V519" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W519" s="9" t="str">
         <x:v>GPAIs can be used to aid in the automated discovery of software vulnerabilities [33].</x:v>
@@ -44536,7 +44536,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V520" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W520" s="9" t="str">
         <x:v>… infrastructure damage - Damage, disruption to or destruction of systems essential to the functioning and safety of a nation or state, including energy, transport …</x:v>
@@ -44788,7 +44788,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V523" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W523" s="9" t="str">
         <x:v>GPAI models are often easily reconfigured for various use cases or have competencies beyond the intended use [78, 225].</x:v>
@@ -44954,7 +44954,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V525" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W525" s="9" t="str">
         <x:v>In other words, agents can be considered vulnerable extensions of their principals, introducing a novel attack surface (SecureWorks, 2023).</x:v>
@@ -45038,7 +45038,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V526" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W526" s="9" t="str">
         <x:v>Various new or existing text encodings, such as Base64, can be employed to craft jailbreak attacks that bypass safety training [13].</x:v>
@@ -45122,7 +45122,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V527" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W527" s="9" t="str">
         <x:v>… gen- erated automatically in a “white box” setting, where access to internal training parameters is required for creation and optimization of the attack [238].</x:v>
@@ -45206,7 +45206,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V528" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W528" s="9" t="str">
         <x:v>… actors such as foreign actors can use such systems to cause large damage if they gain unrestricted or unmonitored access to those AI systems.</x:v>
@@ -45294,7 +45294,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V529" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W529" s="9" t="str">
         <x:v>The growing integration and interconnectivity with external tools and plugins increase the risk of exposure to malicious external inputs.</x:v>
@@ -45378,7 +45378,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V530" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W530" s="9" t="str">
         <x:v>A jailbreak is a type of adversarial input to the model (during deployment) re- sulting in model behavior deviating from intended use.</x:v>
@@ -45462,7 +45462,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V531" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W531" s="9" t="str">
         <x:v>Generative models can create harmful or discriminatory content from benign user requests.</x:v>
@@ -45546,7 +45546,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V532" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W532" s="9" t="str">
         <x:v>… as attacks on overseer agents (see Case Study 13), attempts to thwart cooperation (Huang et al., 2024; Lamport et al., 1982), and the leakage …</x:v>
@@ -45630,7 +45630,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V533" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W533" s="9" t="str">
         <x:v>… in a model’s architec- tures that have no separation between system instructions and user data to produce a harmful output (Perez and Ribeiro, 2022).</x:v>
@@ -45714,7 +45714,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2502.14143</x:v>
       </x:c>
       <x:c r="V534" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2502.14143</x:v>
+        <x:v>https://arxiv.org/pdf/2502.14143</x:v>
       </x:c>
       <x:c r="W534" s="9" t="str">
         <x:v>… to thwart cooperation (Huang et al., 2024; Lamport et al., 1982), and the leakage of information (accidentally or deliberately) that could be used to …</x:v>
@@ -45798,7 +45798,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V535" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W535" s="9" t="str">
         <x:v>… difference is that prompt injections and adversarial inputs usually seek to steer the model towards producing harmful or incorrect outputs from one query, whereas …</x:v>
@@ -45882,7 +45882,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V536" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W536" s="9" t="str">
         <x:v>… be more likely to produce undesired or harmful outputs (as compared to the non-fine-tuned model), even if the fine-tuning was done with harmless and …</x:v>
@@ -46380,7 +46380,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V542" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W542" s="9" t="str">
         <x:v>… inter- pretability could be used to identify neurons responsible for specific functions, and certain neurons that encode safety-related features may be modified to de- …</x:v>
@@ -46638,7 +46638,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V545" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W545" s="9" t="str">
         <x:v>… sensitive or prohibitive attributes, such as race or gender, and instead include desired attributes, even though they do not accurately represent the underlying model.</x:v>
@@ -46722,7 +46722,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V546" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W546" s="9" t="str">
         <x:v>This can lead to a false sense of safety and trust due to a lack of understanding of the model’s limitations.</x:v>
@@ -46806,7 +46806,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V547" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W547" s="9" t="str">
         <x:v>… in schema by a collaborating party can result in an unusable dataset and wasted data collection efforts, or it can lead to misunderstandings about …</x:v>
@@ -46890,7 +46890,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V548" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W548" s="9" t="str">
         <x:v>Models can employ steganography techniques to encode their intermediate rea- soning steps in ways that are not interpretable by humans [166].</x:v>
@@ -47308,7 +47308,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V553" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W553" s="9" t="str">
         <x:v>Chain-of-thought reasoning is sometimes employed to get a better understanding of the model’s output, where it encourages transparent reasoning in text form.</x:v>
@@ -47558,7 +47558,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V556" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W556" s="9" t="str">
         <x:v>When multiple actors are involved in AI development and deployment, it becomes difficult to assign responsibility for harm, complicating accountability.</x:v>
@@ -47808,7 +47808,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V559" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W559" s="9" t="str">
         <x:v>The results of explainability techniques are not free of bias and require careful interpretation.</x:v>
@@ -49224,7 +49224,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2407.01294</x:v>
       </x:c>
       <x:c r="V576" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2407.01294</x:v>
+        <x:v>https://arxiv.org/pdf/2407.01294</x:v>
       </x:c>
       <x:c r="W576" s="9" t="str">
         <x:v>… - Physical pain, injury, illness, or disease suffered by an individual or group due to the malfunction, use or misuse of a technology system.</x:v>
@@ -49398,7 +49398,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2406.13843</x:v>
       </x:c>
       <x:c r="V578" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2406.13843</x:v>
+        <x:v>https://arxiv.org/pdf/2406.13843</x:v>
       </x:c>
       <x:c r="W578" s="9" t="str">
         <x:v>Privacy Compromise attacks reveal sensitive or private information that was used to train a model.</x:v>
@@ -49900,7 +49900,7 @@
         <x:v>10.48550/arXiv.1511.03246</x:v>
       </x:c>
       <x:c r="V584" s="9" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.1511.03246</x:v>
+        <x:v>https://arxiv.org/pdf/1511.03246</x:v>
       </x:c>
       <x:c r="W584" s="9" t="str">
         <x:v>… logical) in the source code, disproportionate weights in the fitness function, or goals misaligned with human values leading to complete disregard for human safety.</x:v>
@@ -49984,7 +49984,7 @@
         <x:v>https://doi.org/10.48550/arXiv.2410.23472</x:v>
       </x:c>
       <x:c r="V585" s="9" t="str">
-        <x:v>https://arxiv.org/abs/2410.23472</x:v>
+        <x:v>https://arxiv.org/pdf/2410.23472</x:v>
       </x:c>
       <x:c r="W585" s="9" t="str">
         <x:v>This usually involves AI systems working in undigitized and physical environments.</x:v>
@@ -52130,7 +52130,7 @@
         <x:v>http://dx.doi.org/10.2139/ssrn.5030173</x:v>
       </x:c>
       <x:c r="V611" s="9" t="str">
-        <x:v>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=5030173</x:v>
+        <x:v>https://arxiv.org/pdf/2412.07780</x:v>
       </x:c>
       <x:c r="W611" s="9" t="str">
         <x:v>The unpredictable trajectory of AI development complicates governance and risk management.</x:v>
@@ -52544,7 +52544,7 @@
         <x:v>10.48550/arXiv.1511.03246</x:v>
       </x:c>
       <x:c r="V616" s="9" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.1511.03246</x:v>
+        <x:v>https://arxiv.org/pdf/1511.03246</x:v>
       </x:c>
       <x:c r="W616" s="9" t="str">
         <x:v>… individual bits may be flipped in different hardware devices due to manufacturing defects or cosmic rays hitting just the right spot (Simonite March 7 …</x:v>

</xml_diff>